<commit_message>
Final PED v3.0, Prod smoke tests (7 of 7 Pass), k6 stress results and ERD v3
</commit_message>
<xml_diff>
--- a/docs/CivicConnect manual test log.xlsx
+++ b/docs/CivicConnect manual test log.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -173,9 +173,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -184,6 +181,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -586,7 +586,11 @@
           <t>Prod URL</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>https://civicconnect-pxjj.onrender.com</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -594,7 +598,11 @@
           <t>Prod commit</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -628,7 +636,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>main 6a198c4 = prod a21dac1. The later fix/m3-review-cleanup commit changes only a log line, tests and documents (no UI or API change), so these results also apply to it.</t>
+          <t>Test build: main 6a198c4 = prod a21dac1. Prod sheet: prod 3bb0a3e (v3.0.0-rc1). The changes after a21dac1 (fix/m3-review-cleanup) touch only a log line, tests and documents (no UI or API change), so the test-build results also apply to the release candidate.</t>
         </is>
       </c>
     </row>
@@ -979,7 +987,7 @@
           <t>Each lands on their own home page and sees only their own menu items.</t>
         </is>
       </c>
-      <c r="G6" s="21" t="inlineStr">
+      <c r="G6" s="20" t="inlineStr">
         <is>
           <t>Thabo on requester page (My Requests, New Request, Profile), Ayesha on staff queue (Requests, My account), Lerato on management (Activity, Requests, Categories, Staff, Audit, My account). Each only own menu.</t>
         </is>
@@ -989,22 +997,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I6" s="23" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J6" s="21" t="inlineStr">
+      <c r="J6" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K6" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L6" s="21" t="inlineStr">
+      <c r="K6" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1041,7 +1049,7 @@
           <t>An error message shows; you stay on the login page, logged out.</t>
         </is>
       </c>
-      <c r="G7" s="21" t="inlineStr">
+      <c r="G7" s="20" t="inlineStr">
         <is>
           <t>Error message shown, stayed on login page, not logged in.</t>
         </is>
@@ -1051,22 +1059,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I7" s="23" t="inlineStr">
+      <c r="I7" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J7" s="21" t="inlineStr">
+      <c r="J7" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K7" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L7" s="21" t="inlineStr">
+      <c r="K7" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L7" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1103,7 +1111,7 @@
           <t>The 6th attempt shows the "too many attempts" message. Wait for the lockout to end before reusing the account.</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
+      <c r="G8" s="20" t="inlineStr">
         <is>
           <t>After 5 failed logins the 6th attempt showed the too many attempts message.</t>
         </is>
@@ -1113,22 +1121,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I8" s="21" t="inlineStr">
+      <c r="I8" s="20" t="inlineStr">
         <is>
           <t>Used pieter.smit (spare account)</t>
         </is>
       </c>
-      <c r="J8" s="21" t="inlineStr">
+      <c r="J8" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K8" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L8" s="21" t="inlineStr">
+      <c r="K8" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1165,7 +1173,7 @@
           <t>You are sent to the login page; no request data shows.</t>
         </is>
       </c>
-      <c r="G9" s="21" t="inlineStr">
+      <c r="G9" s="20" t="inlineStr">
         <is>
           <t>After logout, Back and opening /staff/requests both sent me to login, no request data shown.</t>
         </is>
@@ -1175,22 +1183,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I9" s="23" t="inlineStr">
+      <c r="I9" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J9" s="21" t="inlineStr">
+      <c r="J9" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K9" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L9" s="21" t="inlineStr">
+      <c r="K9" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L9" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1227,7 +1235,7 @@
           <t>You are sent away from the page; no staff or management data shows.</t>
         </is>
       </c>
-      <c r="G10" s="21" t="inlineStr">
+      <c r="G10" s="20" t="inlineStr">
         <is>
           <t>As requester, /management/staff and /staff/requests both redirected away, no staff or management data shown.</t>
         </is>
@@ -1237,22 +1245,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I10" s="23" t="inlineStr">
+      <c r="I10" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J10" s="21" t="inlineStr">
+      <c r="J10" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K10" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L10" s="21" t="inlineStr">
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L10" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1289,7 +1297,7 @@
           <t>The page reloads normally (no 404 or blank page).</t>
         </is>
       </c>
-      <c r="G11" s="21" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>Refreshed /requests/mine, page reloaded normally, no 404 or blank page.</t>
         </is>
@@ -1299,22 +1307,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I11" s="23" t="inlineStr">
+      <c r="I11" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J11" s="21" t="inlineStr">
+      <c r="J11" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K11" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L11" s="21" t="inlineStr">
+      <c r="K11" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L11" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1369,7 +1377,7 @@
           <t>Registration succeeds; login works and shows the requester home page.</t>
         </is>
       </c>
-      <c r="G13" s="21" t="inlineStr">
+      <c r="G13" s="20" t="inlineStr">
         <is>
           <t>Registered cb.test1@example.com, logged in with it, requester home page shown.</t>
         </is>
@@ -1379,22 +1387,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I13" s="23" t="inlineStr">
+      <c r="I13" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J13" s="21" t="inlineStr">
+      <c r="J13" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K13" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L13" s="21" t="inlineStr">
+      <c r="K13" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L13" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1431,7 +1439,7 @@
           <t>Same message as a new registration; the new password does not log in.</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
+      <c r="G14" s="20" t="inlineStr">
         <is>
           <t>Registering with existing email showed the same message as a new registration, new password did not log in.</t>
         </is>
@@ -1441,22 +1449,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I14" s="21" t="inlineStr">
+      <c r="I14" s="20" t="inlineStr">
         <is>
           <t>Used fatima.adams.</t>
         </is>
       </c>
-      <c r="J14" s="21" t="inlineStr">
+      <c r="J14" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K14" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L14" s="21" t="inlineStr">
+      <c r="K14" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L14" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1493,7 +1501,7 @@
           <t>Validation messages show next to the fields; no request is created.</t>
         </is>
       </c>
-      <c r="G15" s="21" t="inlineStr">
+      <c r="G15" s="20" t="inlineStr">
         <is>
           <t>Validation messages shown next to each required field, no request created.</t>
         </is>
@@ -1503,22 +1511,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I15" s="23" t="inlineStr">
+      <c r="I15" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J15" s="21" t="inlineStr">
+      <c r="J15" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K15" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L15" s="21" t="inlineStr">
+      <c r="K15" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L15" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1555,7 +1563,7 @@
           <t>Confirmation with a reference CC-yyyy-nnnnnn and status New; the request is at the top of My Requests.</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
+      <c r="G16" s="20" t="inlineStr">
         <is>
           <t>Confirmation with reference CC-2026-000020 and status New, request at top of My requests.</t>
         </is>
@@ -1565,22 +1573,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I16" s="23" t="inlineStr">
+      <c r="I16" s="22" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="J16" s="21" t="inlineStr">
+      <c r="J16" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K16" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L16" s="21" t="inlineStr">
+      <c r="K16" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1617,7 +1625,7 @@
           <t>New status, time and the visible note show; no staff names and no internal note.</t>
         </is>
       </c>
-      <c r="G17" s="21" t="inlineStr">
+      <c r="G17" s="20" t="inlineStr">
         <is>
           <t>Requester saw new status, time and visible note, no staff names and no internal note.</t>
         </is>
@@ -1627,22 +1635,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I17" s="21" t="inlineStr">
+      <c r="I17" s="20" t="inlineStr">
         <is>
           <t>Handler steps done as Ayesha.</t>
         </is>
       </c>
-      <c r="J17" s="21" t="inlineStr">
+      <c r="J17" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K17" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L17" s="21" t="inlineStr">
+      <c r="K17" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L17" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1679,7 +1687,7 @@
           <t>The inactive category is not in the list.</t>
         </is>
       </c>
-      <c r="G18" s="21" t="inlineStr">
+      <c r="G18" s="20" t="inlineStr">
         <is>
           <t>Deactivated category was not in the requester category list.</t>
         </is>
@@ -1689,22 +1697,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I18" s="21" t="inlineStr">
+      <c r="I18" s="20" t="inlineStr">
         <is>
           <t>Used Damaged Equipment. Category reactivated after the test.</t>
         </is>
       </c>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="J18" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K18" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L18" s="21" t="inlineStr">
+      <c r="K18" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1741,7 +1749,7 @@
           <t>Changes are saved; login works with the new email.</t>
         </is>
       </c>
-      <c r="G19" s="21" t="inlineStr">
+      <c r="G19" s="20" t="inlineStr">
         <is>
           <t>Changed name and email on profile, saved, logged in with the new email.</t>
         </is>
@@ -1751,22 +1759,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I19" s="21" t="inlineStr">
+      <c r="I19" s="20" t="inlineStr">
         <is>
           <t>Used zanele.mahlangu.</t>
         </is>
       </c>
-      <c r="J19" s="21" t="inlineStr">
+      <c r="J19" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K19" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L19" s="21" t="inlineStr">
+      <c r="K19" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L19" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1821,7 +1829,7 @@
           <t>Only requests in the handler's own categories are listed.</t>
         </is>
       </c>
-      <c r="G21" s="21" t="inlineStr">
+      <c r="G21" s="20" t="inlineStr">
         <is>
           <t>Queue showed only Damaged Equipment and IT Support requests; CC-2026-000001 (Facility Faults) and CC-2026-000004 (Security Concerns) not listed.</t>
         </is>
@@ -1832,17 +1840,17 @@
         </is>
       </c>
       <c r="I21" s="18" t="n"/>
-      <c r="J21" s="21" t="inlineStr">
+      <c r="J21" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K21" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L21" s="21" t="inlineStr">
+      <c r="K21" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L21" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -1890,12 +1898,12 @@
         </is>
       </c>
       <c r="I22" s="18" t="n"/>
-      <c r="J22" s="21" t="inlineStr">
+      <c r="J22" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K22" s="22" t="inlineStr">
+      <c r="K22" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -1937,7 +1945,7 @@
           <t>It shows as assigned to you, with the time.</t>
         </is>
       </c>
-      <c r="G23" s="21" t="inlineStr">
+      <c r="G23" s="20" t="inlineStr">
         <is>
           <t>Accepted CC-2026-000002: status New → Assigned, handler shown as Ayesha, history shows Ayesha Patel with time.</t>
         </is>
@@ -1948,12 +1956,12 @@
         </is>
       </c>
       <c r="I23" s="18" t="n"/>
-      <c r="J23" s="21" t="inlineStr">
+      <c r="J23" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K23" s="22" t="inlineStr">
+      <c r="K23" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -1995,7 +2003,7 @@
           <t>One succeeds; the other gets an "already assigned" message.</t>
         </is>
       </c>
-      <c r="G24" s="21" t="inlineStr">
+      <c r="G24" s="20" t="inlineStr">
         <is>
           <t>Ayesha and MT Tester both had CC-2026-000021 open and clicked Accept within a second. MT-Tester got it; the other got "This request is already assigned." Only one handler in the history.</t>
         </is>
@@ -2006,12 +2014,12 @@
         </is>
       </c>
       <c r="I24" s="18" t="n"/>
-      <c r="J24" s="21" t="inlineStr">
+      <c r="J24" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K24" s="22" t="inlineStr">
+      <c r="K24" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2053,7 +2061,7 @@
           <t>Only valid next statuses are offered; Update stays disabled until one is chosen.</t>
         </is>
       </c>
-      <c r="G25" s="21" t="inlineStr">
+      <c r="G25" s="20" t="inlineStr">
         <is>
           <t>On assigned request CC-2026-000002, Update was disabled until a status was chosen; only In Progress and Rejected were offered.</t>
         </is>
@@ -2064,12 +2072,12 @@
         </is>
       </c>
       <c r="I25" s="18" t="n"/>
-      <c r="J25" s="21" t="inlineStr">
+      <c r="J25" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K25" s="22" t="inlineStr">
+      <c r="K25" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2122,12 +2130,12 @@
         </is>
       </c>
       <c r="I26" s="18" t="n"/>
-      <c r="J26" s="21" t="inlineStr">
+      <c r="J26" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K26" s="22" t="inlineStr">
+      <c r="K26" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2180,12 +2188,12 @@
         </is>
       </c>
       <c r="I27" s="18" t="n"/>
-      <c r="J27" s="21" t="inlineStr">
+      <c r="J27" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K27" s="22" t="inlineStr">
+      <c r="K27" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2238,12 +2246,12 @@
         </is>
       </c>
       <c r="I28" s="18" t="n"/>
-      <c r="J28" s="21" t="inlineStr">
+      <c r="J28" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K28" s="22" t="inlineStr">
+      <c r="K28" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2296,12 +2304,12 @@
         </is>
       </c>
       <c r="I29" s="18" t="n"/>
-      <c r="J29" s="21" t="inlineStr">
+      <c r="J29" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K29" s="22" t="inlineStr">
+      <c r="K29" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2361,7 +2369,7 @@
           <t>The handler's list shows High; the history shows who set it.</t>
         </is>
       </c>
-      <c r="G31" s="21" t="inlineStr">
+      <c r="G31" s="20" t="inlineStr">
         <is>
           <t>Lerato set CC-2026-000003 to High on the Activity page ("Priority saved."). Ayesha's queue showed High; history showed "Lerato Nkosi - set the priority to High" with time. Handler cannot change priority.</t>
         </is>
@@ -2372,12 +2380,12 @@
         </is>
       </c>
       <c r="I31" s="18" t="n"/>
-      <c r="J31" s="21" t="inlineStr">
+      <c r="J31" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K31" s="22" t="inlineStr">
+      <c r="K31" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2419,7 +2427,7 @@
           <t>Open, overdue, resolved and closed counts show and match the data.</t>
         </is>
       </c>
-      <c r="G32" s="21" t="inlineStr">
+      <c r="G32" s="20" t="inlineStr">
         <is>
           <t>Activity (last 30 days) showed Open 9, Overdue 4, Resolved 2, Closed 2, Rejected 1. Category rows add up to the tiles; Closed matched the Requests list filtered by Closed (incl. CC-2026-000002); overdue ≤ open.</t>
         </is>
@@ -2430,12 +2438,12 @@
         </is>
       </c>
       <c r="I32" s="18" t="n"/>
-      <c r="J32" s="21" t="inlineStr">
+      <c r="J32" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K32" s="22" t="inlineStr">
+      <c r="K32" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2477,7 +2485,7 @@
           <t>Counts and lists both change to match. (Lists fail until the FR-013 fix.)</t>
         </is>
       </c>
-      <c r="G33" s="21" t="inlineStr">
+      <c r="G33" s="20" t="inlineStr">
         <is>
           <t>Changing category, status and date range each updated both the counts and the request list.</t>
         </is>
@@ -2487,22 +2495,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I33" s="21" t="inlineStr">
+      <c r="I33" s="20" t="inlineStr">
         <is>
           <t>Fixed in PR #32 (D-41).</t>
         </is>
       </c>
-      <c r="J33" s="21" t="inlineStr">
+      <c r="J33" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K33" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L33" s="21" t="inlineStr">
+      <c r="K33" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L33" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -2539,7 +2547,7 @@
           <t>The requester sees the new category, then no longer sees it.</t>
         </is>
       </c>
-      <c r="G34" s="21" t="inlineStr">
+      <c r="G34" s="20" t="inlineStr">
         <is>
           <t>Lerato added "MT-26 test category"; it appeared in Thabo's New request category list. After Deactivate it stayed in the Categories table as Inactive and disappeared from the requester's list (Parking also not offered).</t>
         </is>
@@ -2550,12 +2558,12 @@
         </is>
       </c>
       <c r="I34" s="18" t="n"/>
-      <c r="J34" s="21" t="inlineStr">
+      <c r="J34" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K34" s="22" t="inlineStr">
+      <c r="K34" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2608,12 +2616,12 @@
         </is>
       </c>
       <c r="I35" s="18" t="n"/>
-      <c r="J35" s="21" t="inlineStr">
+      <c r="J35" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K35" s="22" t="inlineStr">
+      <c r="K35" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2655,7 +2663,7 @@
           <t>Handler is logged out on the next action; their open requests go back to the queue.</t>
         </is>
       </c>
-      <c r="G36" s="21" t="inlineStr">
+      <c r="G36" s="20" t="inlineStr">
         <is>
           <t>Lerato deactivated MT Tester while logged in elsewhere. MT Tester's next click went to the login page with an "account no longer active" message; re-login refused. CC-2026-000021 went from Assigned back to New with no handler; history shows removal + internal note by Lerato.</t>
         </is>
@@ -2666,12 +2674,12 @@
         </is>
       </c>
       <c r="I36" s="18" t="n"/>
-      <c r="J36" s="21" t="inlineStr">
+      <c r="J36" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K36" s="22" t="inlineStr">
+      <c r="K36" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2723,17 +2731,17 @@
           <t>Blocked</t>
         </is>
       </c>
-      <c r="I37" s="21" t="inlineStr">
+      <c r="I37" s="20" t="inlineStr">
         <is>
           <t>Covered by automated tests EmployeeServiceTest.lastManagerProtected and ApiHttpIntegrationTest.lastManagerCannotBeDeactivated (CI, fresh DB). Can be run manually on a local DB with a single manager.</t>
         </is>
       </c>
-      <c r="J37" s="21" t="inlineStr">
+      <c r="J37" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K37" s="22" t="inlineStr">
+      <c r="K37" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2786,12 +2794,12 @@
         </is>
       </c>
       <c r="I38" s="18" t="n"/>
-      <c r="J38" s="21" t="inlineStr">
+      <c r="J38" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K38" s="22" t="inlineStr">
+      <c r="K38" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2851,7 +2859,7 @@
           <t>"Service temporarily unavailable" shows, not a blank page.</t>
         </is>
       </c>
-      <c r="G40" s="21" t="inlineStr">
+      <c r="G40" s="20" t="inlineStr">
         <is>
           <t>Backend running locally, Wi-Fi switched off so the test Supabase DB was unreachable. Requests page showed "Service temporarily unavailable." after ~30 s (connection timeout), no blank page. With Wi-Fi back on, the page loaded normally without a restart.</t>
         </is>
@@ -2866,12 +2874,12 @@
           <t>Simulated by cutting the network instead of stopping the shared DB. ~30 s wait before the message is the Hikari connection timeout.</t>
         </is>
       </c>
-      <c r="J40" s="21" t="inlineStr">
+      <c r="J40" s="20" t="inlineStr">
         <is>
           <t>Eduard Herman</t>
         </is>
       </c>
-      <c r="K40" s="22" t="inlineStr">
+      <c r="K40" s="21" t="inlineStr">
         <is>
           <t>16/10/2026</t>
         </is>
@@ -2913,7 +2921,7 @@
           <t>The details always match the selected request. (Fails until the D-38 fix.)</t>
         </is>
       </c>
-      <c r="G41" s="21" t="inlineStr">
+      <c r="G41" s="20" t="inlineStr">
         <is>
           <t>Clicked quickly between CC-2026-000020 and CC-2026-000013 about 10 times, details always matched the selected request.</t>
         </is>
@@ -2923,22 +2931,22 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="I41" s="21" t="inlineStr">
+      <c r="I41" s="20" t="inlineStr">
         <is>
           <t>Fixed in PR #32 (D-38).</t>
         </is>
       </c>
-      <c r="J41" s="21" t="inlineStr">
+      <c r="J41" s="20" t="inlineStr">
         <is>
           <t>Clarissa Bierman</t>
         </is>
       </c>
-      <c r="K41" s="22" t="inlineStr">
-        <is>
-          <t>16/10/2026</t>
-        </is>
-      </c>
-      <c r="L41" s="21" t="inlineStr">
+      <c r="K41" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L41" s="20" t="inlineStr">
         <is>
           <t>a21dac1</t>
         </is>
@@ -3001,7 +3009,7 @@
       </c>
       <c r="I43" s="18" t="n"/>
       <c r="J43" s="18" t="n"/>
-      <c r="K43" s="19" t="n"/>
+      <c r="K43" s="23" t="n"/>
       <c r="L43" s="18" t="n"/>
     </row>
   </sheetData>
@@ -3143,7 +3151,7 @@
       <c r="K5" s="16" t="n"/>
       <c r="L5" s="16" t="n"/>
     </row>
-    <row r="6">
+    <row r="6" ht="25.5" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>P-01</t>
@@ -3174,18 +3182,38 @@
           <t>Shows {"database":"UP","status":"UP"}.</t>
         </is>
       </c>
-      <c r="G6" s="18" t="n"/>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Showed {"database":"UP","status":"UP"}</t>
+        </is>
+      </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I6" s="18" t="n"/>
-      <c r="J6" s="18" t="n"/>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="18" t="n"/>
-    </row>
-    <row r="7">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L6" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="25.5" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>P-02</t>
@@ -3212,16 +3240,36 @@
           <t>Loads over HTTPS; refresh works.</t>
         </is>
       </c>
-      <c r="G7" s="18" t="n"/>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>Loaded over HTTPS, refresh on /login worked, no 404</t>
+        </is>
+      </c>
       <c r="H7" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="19" t="n"/>
-      <c r="L7" s="18" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K7" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L7" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="25.5" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
@@ -3250,16 +3298,36 @@
           <t>Both refused; no dummy account exists on prod.</t>
         </is>
       </c>
-      <c r="G8" s="18" t="n"/>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>Both refused, no dummy accounts on prod</t>
+        </is>
+      </c>
       <c r="H8" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="19" t="n"/>
-      <c r="L8" s="18" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K8" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L8" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="25.5" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
@@ -3292,16 +3360,36 @@
           <t>Password changed; log in again with the new one.</t>
         </is>
       </c>
-      <c r="G9" s="18" t="n"/>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>Changed temporary password on My account, logged in with the new one.</t>
+        </is>
+      </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="n"/>
-      <c r="J9" s="18" t="n"/>
-      <c r="K9" s="19" t="n"/>
-      <c r="L9" s="18" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K9" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L9" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="25.5" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
@@ -3334,18 +3422,38 @@
           <t>All load; the 7 categories are listed.</t>
         </is>
       </c>
-      <c r="G10" s="18" t="n"/>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Activity, Categories and Staff all loaded, 7 categories listed.</t>
+        </is>
+      </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I10" s="18" t="n"/>
-      <c r="J10" s="18" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="18" t="n"/>
-    </row>
-    <row r="11">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L10" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="25.5" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>P-06</t>
@@ -3376,18 +3484,38 @@
           <t>You are sent to the login page.</t>
         </is>
       </c>
-      <c r="G11" s="18" t="n"/>
+      <c r="G11" s="20" t="inlineStr">
+        <is>
+          <t>Sent to the login page, no staff data shown.</t>
+        </is>
+      </c>
       <c r="H11" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="18" t="n"/>
-      <c r="K11" s="19" t="n"/>
-      <c r="L11" s="18" t="n"/>
-    </row>
-    <row r="12">
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K11" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L11" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>P-07</t>
@@ -3418,19 +3546,39 @@
           <t>It wakes and works within a minute or two.</t>
         </is>
       </c>
-      <c r="G12" s="18" t="n"/>
+      <c r="G12" s="20" t="inlineStr">
+        <is>
+          <t>Site was idle, loaded after about 90 seconds and worked normally.</t>
+        </is>
+      </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>Not run</t>
-        </is>
-      </c>
-      <c r="I12" s="18" t="n"/>
-      <c r="J12" s="18" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" s="18" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I12" s="22" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>Clarissa Bierman</t>
+        </is>
+      </c>
+      <c r="K12" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="L12" s="18" t="inlineStr">
+        <is>
+          <t>3bb0a3e</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>Never on prod</t>
         </is>

</xml_diff>